<commit_message>
harden: shared engine + template self-check + tests/CI + sanitized template
Addresses the devil's-advocate review:
- #1 drift: extract matkalasku_core.py (config-agnostic engine); matkalasku.py is now a
  thin .env front-end. The same core + xlsx_fill power convey too, kept byte-identical.
- #2 silent wrong-cell fill: verify_template() reads label cells (A3≈Nimi, C9≈Reitti…)
  and REFUSES to fill a template that doesn't match its profile (--no-verify to bypass).
- #3/#5 tests: 14 unittest tests (incl. a read_cell_text self-closing-cell regression)
  + .github/workflows/test.yml on py3.10/3.12.
- #4 portable date: fi_date() instead of strftime %-d (which breaks on Windows).
- #6 robustness: template font-family clamped to valid (openpyxl reads it now);
  signature auto-fits to the template's row heights (fit_to_rows); rate-provenance +
  OSRM-is-a-hint caveats documented in README.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/matkalasku-2026.xlsx
+++ b/templates/matkalasku-2026.xlsx
@@ -93,7 +93,7 @@
             <sz val="12"/>
             <color rgb="FF000000"/>
             <rFont val="Arial"/>
-            <family val="34"/>
+            <family val="2"/>
           </rPr>
           <t>Käyttöautoedun km-korvaus vuonna 2023: 0,13€ /km</t>
         </r>
@@ -112,7 +112,7 @@
             <sz val="12"/>
             <color rgb="FF000000"/>
             <rFont val="Arial"/>
-            <family val="34"/>
+            <family val="2"/>
           </rPr>
           <t>(vuonna 2022: 0,14€ /km)</t>
         </r>
@@ -1390,7 +1390,7 @@
       <sz val="12"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
-      <family val="34"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>

</xml_diff>